<commit_message>
Fixed leakiness proportion comp
</commit_message>
<xml_diff>
--- a/try.xlsx
+++ b/try.xlsx
@@ -31,10 +31,10 @@
     <t>mean_intensity_f</t>
   </si>
   <si>
-    <t>fraction_1</t>
+    <t>fraction_bdy_p</t>
   </si>
   <si>
-    <t>fraction_2</t>
+    <t>fraction_broken_p</t>
   </si>
   <si>
     <t>fraction_3</t>
@@ -43,7 +43,7 @@
     <t>leak_on_bdy</t>
   </si>
   <si>
-    <t>leak_on_broke</t>
+    <t>leak_on_broken</t>
   </si>
   <si>
     <t>centroid_x</t>
@@ -898,7 +898,7 @@
         <v>0</v>
       </c>
       <c r="J10">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="K10">
         <v>0</v>
@@ -1348,7 +1348,7 @@
         <v>0</v>
       </c>
       <c r="J19">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="K19">
         <v>0</v>
@@ -1698,10 +1698,10 @@
         <v>0</v>
       </c>
       <c r="J26">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="K26">
-        <v>0.04</v>
+        <v>0.09</v>
       </c>
       <c r="L26">
         <v>1207.12</v>
@@ -1798,10 +1798,10 @@
         <v>0</v>
       </c>
       <c r="J28">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="K28">
-        <v>0.07000000000000001</v>
+        <v>0.15</v>
       </c>
       <c r="L28">
         <v>1205.49</v>
@@ -1948,10 +1948,10 @@
         <v>0</v>
       </c>
       <c r="J31">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="K31">
-        <v>0.03</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="L31">
         <v>1328.92</v>
@@ -1998,7 +1998,7 @@
         <v>0</v>
       </c>
       <c r="J32">
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="K32">
         <v>0</v>
@@ -2148,10 +2148,10 @@
         <v>0</v>
       </c>
       <c r="J35">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="K35">
-        <v>0.03</v>
+        <v>0.06</v>
       </c>
       <c r="L35">
         <v>161.55</v>
@@ -2848,7 +2848,7 @@
         <v>0</v>
       </c>
       <c r="J49">
-        <v>0.02</v>
+        <v>0.05</v>
       </c>
       <c r="K49">
         <v>0</v>
@@ -2898,10 +2898,10 @@
         <v>0</v>
       </c>
       <c r="J50">
-        <v>0.05</v>
+        <v>0.11</v>
       </c>
       <c r="K50">
-        <v>0.12</v>
+        <v>0.28</v>
       </c>
       <c r="L50">
         <v>882.0599999999999</v>
@@ -3548,10 +3548,10 @@
         <v>0</v>
       </c>
       <c r="J63">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="K63">
-        <v>0.05</v>
+        <v>0.12</v>
       </c>
       <c r="L63">
         <v>88.13</v>
@@ -4048,7 +4048,7 @@
         <v>0</v>
       </c>
       <c r="J73">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="K73">
         <v>0</v>
@@ -4198,7 +4198,7 @@
         <v>0</v>
       </c>
       <c r="J76">
-        <v>0.05</v>
+        <v>0.11</v>
       </c>
       <c r="K76">
         <v>0</v>
@@ -4548,7 +4548,7 @@
         <v>0</v>
       </c>
       <c r="J83">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="K83">
         <v>0</v>
@@ -4648,7 +4648,7 @@
         <v>0</v>
       </c>
       <c r="J85">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="K85">
         <v>0</v>
@@ -4748,7 +4748,7 @@
         <v>0</v>
       </c>
       <c r="J87">
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
       <c r="K87">
         <v>0</v>
@@ -5098,10 +5098,10 @@
         <v>0</v>
       </c>
       <c r="J94">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="K94">
-        <v>0.06</v>
+        <v>0.14</v>
       </c>
       <c r="L94">
         <v>600.59</v>
@@ -5148,10 +5148,10 @@
         <v>0</v>
       </c>
       <c r="J95">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="K95">
-        <v>0.11</v>
+        <v>0.26</v>
       </c>
       <c r="L95">
         <v>190.07</v>
@@ -5198,10 +5198,10 @@
         <v>0</v>
       </c>
       <c r="J96">
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
       <c r="K96">
-        <v>0.13</v>
+        <v>0.32</v>
       </c>
       <c r="L96">
         <v>248.98</v>
@@ -5248,7 +5248,7 @@
         <v>0</v>
       </c>
       <c r="J97">
-        <v>0.03</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="K97">
         <v>0</v>
@@ -5348,10 +5348,10 @@
         <v>0</v>
       </c>
       <c r="J99">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="K99">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
       <c r="L99">
         <v>600.64</v>
@@ -5448,10 +5448,10 @@
         <v>0</v>
       </c>
       <c r="J101">
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
       <c r="K101">
-        <v>0.11</v>
+        <v>0.25</v>
       </c>
       <c r="L101">
         <v>459.54</v>
@@ -5498,7 +5498,7 @@
         <v>0</v>
       </c>
       <c r="J102">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="K102">
         <v>0</v>
@@ -5548,10 +5548,10 @@
         <v>0</v>
       </c>
       <c r="J103">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="K103">
-        <v>0.02</v>
+        <v>0.05</v>
       </c>
       <c r="L103">
         <v>785.2</v>
@@ -5648,10 +5648,10 @@
         <v>0</v>
       </c>
       <c r="J105">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="K105">
-        <v>0.02</v>
+        <v>0.05</v>
       </c>
       <c r="L105">
         <v>816.8099999999999</v>
@@ -5848,10 +5848,10 @@
         <v>0</v>
       </c>
       <c r="J109">
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="K109">
-        <v>0.1</v>
+        <v>0.24</v>
       </c>
       <c r="L109">
         <v>959.87</v>
@@ -5948,10 +5948,10 @@
         <v>0</v>
       </c>
       <c r="J111">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="K111">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="L111">
         <v>1105.39</v>
@@ -6048,10 +6048,10 @@
         <v>0</v>
       </c>
       <c r="J113">
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
       <c r="K113">
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="L113">
         <v>1356.29</v>
@@ -6101,7 +6101,7 @@
         <v>0</v>
       </c>
       <c r="K114">
-        <v>0.02</v>
+        <v>0.05</v>
       </c>
       <c r="L114">
         <v>1410.74</v>
@@ -6248,10 +6248,10 @@
         <v>0</v>
       </c>
       <c r="J117">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="K117">
-        <v>0.41</v>
+        <v>0.89</v>
       </c>
       <c r="L117">
         <v>89.29000000000001</v>
@@ -6448,10 +6448,10 @@
         <v>0</v>
       </c>
       <c r="J121">
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="K121">
-        <v>0.03</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="L121">
         <v>490.14</v>
@@ -6548,7 +6548,7 @@
         <v>0</v>
       </c>
       <c r="J123">
-        <v>0.03</v>
+        <v>0.06</v>
       </c>
       <c r="K123">
         <v>0</v>
@@ -6848,7 +6848,7 @@
         <v>0</v>
       </c>
       <c r="J129">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="K129">
         <v>0</v>
@@ -7648,10 +7648,10 @@
         <v>0</v>
       </c>
       <c r="J145">
-        <v>0.03</v>
+        <v>0.06</v>
       </c>
       <c r="K145">
-        <v>0.09</v>
+        <v>0.24</v>
       </c>
       <c r="L145">
         <v>486.4</v>
@@ -7698,10 +7698,10 @@
         <v>0</v>
       </c>
       <c r="J146">
+        <v>0.04</v>
+      </c>
+      <c r="K146">
         <v>0.02</v>
-      </c>
-      <c r="K146">
-        <v>0.01</v>
       </c>
       <c r="L146">
         <v>50.4</v>
@@ -7748,10 +7748,10 @@
         <v>0</v>
       </c>
       <c r="J147">
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
       <c r="K147">
-        <v>0.13</v>
+        <v>0.33</v>
       </c>
       <c r="L147">
         <v>271.75</v>
@@ -7798,10 +7798,10 @@
         <v>0</v>
       </c>
       <c r="J148">
-        <v>0.07000000000000001</v>
+        <v>0.16</v>
       </c>
       <c r="K148">
-        <v>0.14</v>
+        <v>0.35</v>
       </c>
       <c r="L148">
         <v>655.85</v>
@@ -7848,10 +7848,10 @@
         <v>0</v>
       </c>
       <c r="J149">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="K149">
-        <v>0.16</v>
+        <v>0.41</v>
       </c>
       <c r="L149">
         <v>533.5599999999999</v>
@@ -7898,10 +7898,10 @@
         <v>0</v>
       </c>
       <c r="J150">
-        <v>0.17</v>
+        <v>0.39</v>
       </c>
       <c r="K150">
-        <v>0.33</v>
+        <v>0.82</v>
       </c>
       <c r="L150">
         <v>550.02</v>
@@ -7951,7 +7951,7 @@
         <v>0</v>
       </c>
       <c r="K151">
-        <v>0.16</v>
+        <v>0.4</v>
       </c>
       <c r="L151">
         <v>708.35</v>
@@ -7998,10 +7998,10 @@
         <v>0</v>
       </c>
       <c r="J152">
-        <v>0.08</v>
+        <v>0.19</v>
       </c>
       <c r="K152">
-        <v>0.13</v>
+        <v>0.32</v>
       </c>
       <c r="L152">
         <v>832.67</v>
@@ -8051,7 +8051,7 @@
         <v>0</v>
       </c>
       <c r="K153">
-        <v>0.1</v>
+        <v>0.28</v>
       </c>
       <c r="L153">
         <v>935.74</v>
@@ -8101,7 +8101,7 @@
         <v>0</v>
       </c>
       <c r="K154">
-        <v>0.12</v>
+        <v>0.31</v>
       </c>
       <c r="L154">
         <v>1292.79</v>
@@ -8148,10 +8148,10 @@
         <v>0</v>
       </c>
       <c r="J155">
-        <v>0.06</v>
+        <v>0.14</v>
       </c>
       <c r="K155">
-        <v>0.23</v>
+        <v>0.58</v>
       </c>
       <c r="L155">
         <v>1116.52</v>
@@ -8198,10 +8198,10 @@
         <v>0</v>
       </c>
       <c r="J156">
-        <v>0.07000000000000001</v>
+        <v>0.16</v>
       </c>
       <c r="K156">
-        <v>0.19</v>
+        <v>0.47</v>
       </c>
       <c r="L156">
         <v>1291.58</v>
@@ -8251,7 +8251,7 @@
         <v>0</v>
       </c>
       <c r="K157">
-        <v>0.03</v>
+        <v>0.08</v>
       </c>
       <c r="L157">
         <v>1418.48</v>
@@ -8298,10 +8298,10 @@
         <v>0</v>
       </c>
       <c r="J158">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="K158">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="L158">
         <v>1479.43</v>
@@ -8348,10 +8348,10 @@
         <v>0</v>
       </c>
       <c r="J159">
-        <v>0.07000000000000001</v>
+        <v>0.18</v>
       </c>
       <c r="K159">
-        <v>0.14</v>
+        <v>0.35</v>
       </c>
       <c r="L159">
         <v>1479.19</v>
@@ -8398,10 +8398,10 @@
         <v>0</v>
       </c>
       <c r="J160">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="K160">
-        <v>0.08</v>
+        <v>0.21</v>
       </c>
       <c r="L160">
         <v>175.55</v>
@@ -8448,10 +8448,10 @@
         <v>0</v>
       </c>
       <c r="J161">
-        <v>0.05</v>
+        <v>0.13</v>
       </c>
       <c r="K161">
-        <v>0.14</v>
+        <v>0.34</v>
       </c>
       <c r="L161">
         <v>160.8</v>
@@ -8498,10 +8498,10 @@
         <v>0</v>
       </c>
       <c r="J162">
-        <v>0.02</v>
+        <v>0.05</v>
       </c>
       <c r="K162">
-        <v>0.15</v>
+        <v>0.4</v>
       </c>
       <c r="L162">
         <v>205.29</v>
@@ -8548,10 +8548,10 @@
         <v>0</v>
       </c>
       <c r="J163">
-        <v>0.08</v>
+        <v>0.19</v>
       </c>
       <c r="K163">
-        <v>0.18</v>
+        <v>0.45</v>
       </c>
       <c r="L163">
         <v>42.2</v>
@@ -8598,10 +8598,10 @@
         <v>0</v>
       </c>
       <c r="J164">
-        <v>0.07000000000000001</v>
+        <v>0.17</v>
       </c>
       <c r="K164">
-        <v>0.11</v>
+        <v>0.26</v>
       </c>
       <c r="L164">
         <v>404.03</v>
@@ -8648,10 +8648,10 @@
         <v>0</v>
       </c>
       <c r="J165">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="K165">
-        <v>0.23</v>
+        <v>0.62</v>
       </c>
       <c r="L165">
         <v>471.35</v>
@@ -8698,10 +8698,10 @@
         <v>0</v>
       </c>
       <c r="J166">
-        <v>0.09</v>
+        <v>0.22</v>
       </c>
       <c r="K166">
-        <v>0.15</v>
+        <v>0.39</v>
       </c>
       <c r="L166">
         <v>615.87</v>
@@ -8748,10 +8748,10 @@
         <v>0</v>
       </c>
       <c r="J167">
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
       <c r="K167">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="L167">
         <v>689.09</v>
@@ -8801,7 +8801,7 @@
         <v>0</v>
       </c>
       <c r="K168">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="L168">
         <v>509.96</v>
@@ -8848,10 +8848,10 @@
         <v>0</v>
       </c>
       <c r="J169">
-        <v>0.07000000000000001</v>
+        <v>0.16</v>
       </c>
       <c r="K169">
-        <v>0.22</v>
+        <v>0.57</v>
       </c>
       <c r="L169">
         <v>944.33</v>
@@ -8898,10 +8898,10 @@
         <v>0</v>
       </c>
       <c r="J170">
-        <v>0.09</v>
+        <v>0.22</v>
       </c>
       <c r="K170">
-        <v>0.14</v>
+        <v>0.35</v>
       </c>
       <c r="L170">
         <v>864.24</v>
@@ -8948,10 +8948,10 @@
         <v>0</v>
       </c>
       <c r="J171">
-        <v>0.04</v>
+        <v>0.09</v>
       </c>
       <c r="K171">
-        <v>0.06</v>
+        <v>0.15</v>
       </c>
       <c r="L171">
         <v>1187.75</v>
@@ -8998,10 +8998,10 @@
         <v>0</v>
       </c>
       <c r="J172">
-        <v>0.04</v>
+        <v>0.09</v>
       </c>
       <c r="K172">
-        <v>0.09</v>
+        <v>0.23</v>
       </c>
       <c r="L172">
         <v>1156.94</v>
@@ -9048,10 +9048,10 @@
         <v>0</v>
       </c>
       <c r="J173">
-        <v>0.03</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="K173">
-        <v>0.06</v>
+        <v>0.15</v>
       </c>
       <c r="L173">
         <v>1393.82</v>
@@ -9098,10 +9098,10 @@
         <v>0</v>
       </c>
       <c r="J174">
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="K174">
-        <v>0.06</v>
+        <v>0.15</v>
       </c>
       <c r="L174">
         <v>1496.99</v>
@@ -9201,7 +9201,7 @@
         <v>0</v>
       </c>
       <c r="K176">
-        <v>0.11</v>
+        <v>0.25</v>
       </c>
       <c r="L176">
         <v>168.22</v>
@@ -9248,10 +9248,10 @@
         <v>0</v>
       </c>
       <c r="J177">
-        <v>0.05</v>
+        <v>0.13</v>
       </c>
       <c r="K177">
-        <v>0.11</v>
+        <v>0.27</v>
       </c>
       <c r="L177">
         <v>336.78</v>
@@ -9298,7 +9298,7 @@
         <v>0</v>
       </c>
       <c r="J178">
-        <v>0.02</v>
+        <v>0.05</v>
       </c>
       <c r="K178">
         <v>0.01</v>
@@ -9348,10 +9348,10 @@
         <v>0</v>
       </c>
       <c r="J179">
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="K179">
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="L179">
         <v>218.24</v>
@@ -9401,7 +9401,7 @@
         <v>0.01</v>
       </c>
       <c r="K180">
-        <v>0.06</v>
+        <v>0.14</v>
       </c>
       <c r="L180">
         <v>501.58</v>
@@ -9498,10 +9498,10 @@
         <v>0</v>
       </c>
       <c r="J182">
-        <v>0.05</v>
+        <v>0.11</v>
       </c>
       <c r="K182">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="L182">
         <v>771.37</v>
@@ -9548,10 +9548,10 @@
         <v>0</v>
       </c>
       <c r="J183">
-        <v>0.06</v>
+        <v>0.15</v>
       </c>
       <c r="K183">
-        <v>0.21</v>
+        <v>0.52</v>
       </c>
       <c r="L183">
         <v>809.5599999999999</v>
@@ -9598,10 +9598,10 @@
         <v>0</v>
       </c>
       <c r="J184">
-        <v>0.07000000000000001</v>
+        <v>0.16</v>
       </c>
       <c r="K184">
-        <v>0.14</v>
+        <v>0.36</v>
       </c>
       <c r="L184">
         <v>1076.4</v>
@@ -9648,10 +9648,10 @@
         <v>0</v>
       </c>
       <c r="J185">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="K185">
-        <v>0.12</v>
+        <v>0.29</v>
       </c>
       <c r="L185">
         <v>788.6799999999999</v>
@@ -9698,10 +9698,10 @@
         <v>0</v>
       </c>
       <c r="J186">
-        <v>0.04</v>
+        <v>0.09</v>
       </c>
       <c r="K186">
-        <v>0.1</v>
+        <v>0.26</v>
       </c>
       <c r="L186">
         <v>1162.53</v>
@@ -9748,10 +9748,10 @@
         <v>0</v>
       </c>
       <c r="J187">
-        <v>0.04</v>
+        <v>0.09</v>
       </c>
       <c r="K187">
-        <v>0.16</v>
+        <v>0.39</v>
       </c>
       <c r="L187">
         <v>1096.44</v>
@@ -9801,7 +9801,7 @@
         <v>0</v>
       </c>
       <c r="K188">
-        <v>0.14</v>
+        <v>0.37</v>
       </c>
       <c r="L188">
         <v>1345.22</v>
@@ -9848,10 +9848,10 @@
         <v>0</v>
       </c>
       <c r="J189">
-        <v>0.09</v>
+        <v>0.2</v>
       </c>
       <c r="K189">
-        <v>0.09</v>
+        <v>0.21</v>
       </c>
       <c r="L189">
         <v>1348.5</v>
@@ -9898,10 +9898,10 @@
         <v>0</v>
       </c>
       <c r="J190">
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
       <c r="K190">
-        <v>0.13</v>
+        <v>0.33</v>
       </c>
       <c r="L190">
         <v>1442.74</v>
@@ -9948,10 +9948,10 @@
         <v>0</v>
       </c>
       <c r="J191">
-        <v>0.15</v>
+        <v>0.35</v>
       </c>
       <c r="K191">
-        <v>0.07000000000000001</v>
+        <v>0.16</v>
       </c>
       <c r="L191">
         <v>1495.39</v>
@@ -9998,10 +9998,10 @@
         <v>0</v>
       </c>
       <c r="J192">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="K192">
-        <v>0.07000000000000001</v>
+        <v>0.18</v>
       </c>
       <c r="L192">
         <v>1485.99</v>
@@ -10101,7 +10101,7 @@
         <v>0</v>
       </c>
       <c r="K194">
-        <v>0.13</v>
+        <v>0.3</v>
       </c>
       <c r="L194">
         <v>108.7</v>
@@ -10151,7 +10151,7 @@
         <v>0</v>
       </c>
       <c r="K195">
-        <v>0.14</v>
+        <v>0.37</v>
       </c>
       <c r="L195">
         <v>55.13</v>
@@ -10201,7 +10201,7 @@
         <v>0</v>
       </c>
       <c r="K196">
-        <v>0.09</v>
+        <v>0.23</v>
       </c>
       <c r="L196">
         <v>102.7</v>
@@ -10298,10 +10298,10 @@
         <v>0</v>
       </c>
       <c r="J198">
-        <v>0.03</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="K198">
-        <v>0.15</v>
+        <v>0.39</v>
       </c>
       <c r="L198">
         <v>284.47</v>
@@ -10348,10 +10348,10 @@
         <v>0</v>
       </c>
       <c r="J199">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="K199">
-        <v>0.11</v>
+        <v>0.26</v>
       </c>
       <c r="L199">
         <v>278.29</v>
@@ -10398,10 +10398,10 @@
         <v>0</v>
       </c>
       <c r="J200">
-        <v>0.35</v>
+        <v>0.8</v>
       </c>
       <c r="K200">
-        <v>0.24</v>
+        <v>0.6</v>
       </c>
       <c r="L200">
         <v>415.77</v>
@@ -10451,7 +10451,7 @@
         <v>0</v>
       </c>
       <c r="K201">
-        <v>0.03</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="L201">
         <v>409.81</v>
@@ -10498,10 +10498,10 @@
         <v>0</v>
       </c>
       <c r="J202">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="K202">
-        <v>0.05</v>
+        <v>0.12</v>
       </c>
       <c r="L202">
         <v>598.16</v>
@@ -10548,10 +10548,10 @@
         <v>0</v>
       </c>
       <c r="J203">
-        <v>0.04</v>
+        <v>0.11</v>
       </c>
       <c r="K203">
-        <v>0.09</v>
+        <v>0.24</v>
       </c>
       <c r="L203">
         <v>785.74</v>
@@ -10601,7 +10601,7 @@
         <v>0</v>
       </c>
       <c r="K204">
-        <v>0.13</v>
+        <v>0.3</v>
       </c>
       <c r="L204">
         <v>1066.49</v>
@@ -10648,10 +10648,10 @@
         <v>0</v>
       </c>
       <c r="J205">
-        <v>0.02</v>
+        <v>0.05</v>
       </c>
       <c r="K205">
-        <v>0.11</v>
+        <v>0.27</v>
       </c>
       <c r="L205">
         <v>1344.95</v>
@@ -10698,10 +10698,10 @@
         <v>0</v>
       </c>
       <c r="J206">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="K206">
-        <v>0.06</v>
+        <v>0.14</v>
       </c>
       <c r="L206">
         <v>1322.29</v>
@@ -10748,10 +10748,10 @@
         <v>0</v>
       </c>
       <c r="J207">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="K207">
-        <v>0.12</v>
+        <v>0.3</v>
       </c>
       <c r="L207">
         <v>1133.82</v>
@@ -10801,7 +10801,7 @@
         <v>0</v>
       </c>
       <c r="K208">
-        <v>0.06</v>
+        <v>0.16</v>
       </c>
       <c r="L208">
         <v>1230.56</v>
@@ -10851,7 +10851,7 @@
         <v>0</v>
       </c>
       <c r="K209">
-        <v>0.17</v>
+        <v>0.45</v>
       </c>
       <c r="L209">
         <v>1440.2</v>
@@ -10901,7 +10901,7 @@
         <v>0</v>
       </c>
       <c r="K210">
-        <v>0.25</v>
+        <v>0.65</v>
       </c>
       <c r="L210">
         <v>1534.17</v>
@@ -10951,7 +10951,7 @@
         <v>0</v>
       </c>
       <c r="K211">
-        <v>0.12</v>
+        <v>0.3</v>
       </c>
       <c r="L211">
         <v>121.78</v>
@@ -10998,10 +10998,10 @@
         <v>0</v>
       </c>
       <c r="J212">
-        <v>0.06</v>
+        <v>0.14</v>
       </c>
       <c r="K212">
-        <v>0.2</v>
+        <v>0.49</v>
       </c>
       <c r="L212">
         <v>134.98</v>
@@ -11048,10 +11048,10 @@
         <v>0</v>
       </c>
       <c r="J213">
-        <v>0.05</v>
+        <v>0.12</v>
       </c>
       <c r="K213">
-        <v>0.18</v>
+        <v>0.44</v>
       </c>
       <c r="L213">
         <v>121.94</v>
@@ -11098,10 +11098,10 @@
         <v>0</v>
       </c>
       <c r="J214">
-        <v>0.03</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="K214">
-        <v>0.03</v>
+        <v>0.08</v>
       </c>
       <c r="L214">
         <v>345.25</v>
@@ -11148,10 +11148,10 @@
         <v>0</v>
       </c>
       <c r="J215">
-        <v>0.05</v>
+        <v>0.12</v>
       </c>
       <c r="K215">
-        <v>0.08</v>
+        <v>0.2</v>
       </c>
       <c r="L215">
         <v>50.12</v>
@@ -11248,10 +11248,10 @@
         <v>0</v>
       </c>
       <c r="J217">
-        <v>0.06</v>
+        <v>0.13</v>
       </c>
       <c r="K217">
-        <v>0.21</v>
+        <v>0.51</v>
       </c>
       <c r="L217">
         <v>551.4</v>
@@ -11298,10 +11298,10 @@
         <v>0</v>
       </c>
       <c r="J218">
-        <v>0.02</v>
+        <v>0.05</v>
       </c>
       <c r="K218">
-        <v>0.19</v>
+        <v>0.47</v>
       </c>
       <c r="L218">
         <v>578.77</v>
@@ -11398,10 +11398,10 @@
         <v>0</v>
       </c>
       <c r="J220">
-        <v>0.02</v>
+        <v>0.05</v>
       </c>
       <c r="K220">
-        <v>0.25</v>
+        <v>0.66</v>
       </c>
       <c r="L220">
         <v>732.1</v>
@@ -11448,10 +11448,10 @@
         <v>0</v>
       </c>
       <c r="J221">
-        <v>0.03</v>
+        <v>0.06</v>
       </c>
       <c r="K221">
-        <v>0.14</v>
+        <v>0.37</v>
       </c>
       <c r="L221">
         <v>798.62</v>
@@ -11498,10 +11498,10 @@
         <v>0</v>
       </c>
       <c r="J222">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="K222">
-        <v>0.16</v>
+        <v>0.43</v>
       </c>
       <c r="L222">
         <v>914.34</v>
@@ -11548,10 +11548,10 @@
         <v>0</v>
       </c>
       <c r="J223">
-        <v>0.33</v>
+        <v>0.78</v>
       </c>
       <c r="K223">
-        <v>0.15</v>
+        <v>0.38</v>
       </c>
       <c r="L223">
         <v>989.1900000000001</v>
@@ -11598,10 +11598,10 @@
         <v>0</v>
       </c>
       <c r="J224">
-        <v>0.04</v>
+        <v>0.09</v>
       </c>
       <c r="K224">
-        <v>0.21</v>
+        <v>0.55</v>
       </c>
       <c r="L224">
         <v>1180.33</v>
@@ -11648,10 +11648,10 @@
         <v>0</v>
       </c>
       <c r="J225">
-        <v>0.09</v>
+        <v>0.22</v>
       </c>
       <c r="K225">
-        <v>0.25</v>
+        <v>0.64</v>
       </c>
       <c r="L225">
         <v>1129.89</v>
@@ -11698,10 +11698,10 @@
         <v>0</v>
       </c>
       <c r="J226">
-        <v>0.05</v>
+        <v>0.11</v>
       </c>
       <c r="K226">
-        <v>0.15</v>
+        <v>0.38</v>
       </c>
       <c r="L226">
         <v>1319.11</v>
@@ -11748,10 +11748,10 @@
         <v>0</v>
       </c>
       <c r="J227">
-        <v>0.11</v>
+        <v>0.25</v>
       </c>
       <c r="K227">
-        <v>0.3</v>
+        <v>0.78</v>
       </c>
       <c r="L227">
         <v>1276.15</v>
@@ -11798,10 +11798,10 @@
         <v>0</v>
       </c>
       <c r="J228">
-        <v>0.19</v>
+        <v>0.45</v>
       </c>
       <c r="K228">
-        <v>0.14</v>
+        <v>0.34</v>
       </c>
       <c r="L228">
         <v>1418.01</v>
@@ -11848,10 +11848,10 @@
         <v>0</v>
       </c>
       <c r="J229">
-        <v>0.15</v>
+        <v>0.35</v>
       </c>
       <c r="K229">
-        <v>0.25</v>
+        <v>0.66</v>
       </c>
       <c r="L229">
         <v>1482.43</v>
@@ -11898,10 +11898,10 @@
         <v>0</v>
       </c>
       <c r="J230">
-        <v>0.17</v>
+        <v>0.38</v>
       </c>
       <c r="K230">
-        <v>0.12</v>
+        <v>0.28</v>
       </c>
       <c r="L230">
         <v>1497.48</v>
@@ -11948,10 +11948,10 @@
         <v>0</v>
       </c>
       <c r="J231">
-        <v>0.42</v>
+        <v>1</v>
       </c>
       <c r="K231">
-        <v>0.36</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="L231">
         <v>1536.99</v>

</xml_diff>